<commit_message>
chore: Lectura por familia + hoja Veredicto en xlsx de pegado W33
</commit_message>
<xml_diff>
--- a/pegar-sheet-W33/UPDATE-Sheet-W33.xlsx
+++ b/pegar-sheet-W33/UPDATE-Sheet-W33.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Campanas_ASINs" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Acciones_PPC" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Bitacora" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Veredicto" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -594,6 +595,11 @@
       <c r="E2" t="n">
         <v>476.66</v>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Gama principal: crece y concentra la mayor parte de la facturación. Por cada euro invertido, el retorno está muy por encima del punto de equilibrio.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -613,6 +619,11 @@
       <c r="E3" t="n">
         <v>85.69</v>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Estable dentro del plan acordado. Convierte muy bien, pero se mantiene contenida a propósito por política de margen.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -632,6 +643,11 @@
       <c r="E4" t="n">
         <v>28.45</v>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Estable y contenida, igual que la gama anterior.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -651,6 +667,11 @@
       <c r="E5" t="n">
         <v>40.88</v>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Crece con inversión moderada. Buena señal para reforzar en las próximas semanas.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -670,6 +691,11 @@
       <c r="E6" t="n">
         <v>6.49</v>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Sin ventas esta semana.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -688,6 +714,11 @@
       </c>
       <c r="E7" t="n">
         <v>24.35</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Sin ventas esta semana.</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -2485,4 +2516,82 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Que_pasa</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Cuello</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Palanca</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Bloquea</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>14-ago</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Semana de crecimiento sostenido por conversión</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>La facturación crece frente a la semana anterior. El motor no fue más tráfico sino que quien llega compra más: la gama principal sostiene el volumen y mejora su conversión.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>La visibilidad de la semana se contrajo respecto a la anterior. Ya estamos analizando las posibles causas para confirmar si es estacional o requiere acción; lo cerramos la semana próxima.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Concentrar la inversión en las ubicaciones de mejor retorno y reforzar la gama que viene creciendo.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: Fecha en formato ISO en Acciones_PPC y Bitacora (weekOf del dashboard exige YYYY-MM-DD)
</commit_message>
<xml_diff>
--- a/pegar-sheet-W33/UPDATE-Sheet-W33.xlsx
+++ b/pegar-sheet-W33/UPDATE-Sheet-W33.xlsx
@@ -1600,7 +1600,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>10-ago</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1662,7 +1662,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>10-ago</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1724,7 +1724,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>10-ago</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1786,7 +1786,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>10-ago</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1848,7 +1848,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>10-ago</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1910,7 +1910,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>10-ago</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1972,7 +1972,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>10-ago</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2034,7 +2034,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>10-ago</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2096,7 +2096,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>14-ago</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2158,7 +2158,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>14-ago</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2220,7 +2220,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>14-ago</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2282,7 +2282,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>14-ago</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2344,7 +2344,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>14-ago</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2406,7 +2406,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>14-ago</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2499,7 +2499,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14-ago</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
fix: bloque Acciones_PPC completo 20 filas (13 internas + 7 cliente) + apostrofo en celdas +N%
</commit_message>
<xml_diff>
--- a/pegar-sheet-W33/UPDATE-Sheet-W33.xlsx
+++ b/pegar-sheet-W33/UPDATE-Sheet-W33.xlsx
@@ -51,8 +51,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1532,7 +1533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1638,7 +1639,7 @@
           <t>0%</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>+40%</t>
         </is>
@@ -1700,7 +1701,7 @@
           <t>0%</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="1" t="inlineStr">
         <is>
           <t>+40%</t>
         </is>
@@ -1762,7 +1763,7 @@
           <t>0%</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="1" t="inlineStr">
         <is>
           <t>+25%</t>
         </is>
@@ -1824,7 +1825,7 @@
           <t>0%</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="1" t="inlineStr">
         <is>
           <t>+40%</t>
         </is>
@@ -1881,12 +1882,12 @@
           <t>Modificador Top of Search</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="1" t="inlineStr">
         <is>
           <t>+201%</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="1" t="inlineStr">
         <is>
           <t>+100%</t>
         </is>
@@ -1943,12 +1944,12 @@
           <t>Modificador Top of Search</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="1" t="inlineStr">
         <is>
           <t>+101%</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="1" t="inlineStr">
         <is>
           <t>+50%</t>
         </is>
@@ -2039,7 +2040,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Conjunto de campañas de búsqueda</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2047,11 +2048,6 @@
           <t>Reorientación de inversión hacia posiciones de mejor retorno</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>Se concentró la inversión en las ubicaciones de búsqueda que mejor retorno vienen dando y se contuvo el gasto en las gamas fuera del plan acordado, sin sumar inversión nueva.</t>
@@ -2062,29 +2058,9 @@
           <t>Hecho</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>Se mide a partir de la próxima semana</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>—</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -2096,186 +2072,111 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>4 campañas</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Reallocation ToS → RoS</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Refuerzo de visibilidad en la gama principal</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4 campañas movidas a RoS +40/+25%. Medir efecto a +7d.</t>
+          <t>Ahí cada euro devuelve 10,39 € frente a 7,04 € en la parte superior de la página, y queda inventario sin usar.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Guard vence 17-ago</t>
+          <t>Se mide a partir de la próxima semana</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>interno</t>
+          <t>cliente</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2 campañas</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Contención Moon/Orbit · escalón 2</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Contención de gasto en gamas fuera de plan</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>AUTOSeg +100%→+50% · AUTOBulk +50%→+25%, si el escalón 1 contuvo sin frenar las permitidas.</t>
+          <t>Concentraban inversión en dos líneas que convierten bien pero quedan fuera del plan acordado. Primer escalón de dos.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Depende del veredicto del guard del 17-ago</t>
+          <t>Se mide a partir de la próxima semana</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>interno</t>
+          <t>cliente</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1 campaña</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AMC (Amazon Marketing Cloud)</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Pausa de campaña de recuperación sin retorno</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Pedido de Roger en la meet: segmentación de audiencias. Instancia sin confirmar.</t>
+          <t>112 visitas de pago sin una sola venta. La ficha está activa, así que no es un problema de disponibilidad.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Resolvería el fallo del remarketing genérico</t>
+          <t>Se mide a partir de la próxima semana</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>interno</t>
+          <t>cliente</t>
         </is>
       </c>
     </row>
@@ -2292,7 +2193,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>5 keywords de test</t>
+          <t>Reallocation ToS → RoS</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2302,7 +2203,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>NO LANZADAS. De 26 clusters solo 3 quedaron limpios y son débiles (SV 843-2.419).</t>
+          <t>4 campañas movidas a RoS +40/+25%. Medir efecto a +7d.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -2332,7 +2233,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Diferido hasta refrescar el banco contra el bulk</t>
+          <t>Guard vence 17-ago</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -2354,7 +2255,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BLOCKER · margen real</t>
+          <t>Contención Moon/Orbit · escalón 2</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2364,7 +2265,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Flete FBM no cargado por SKU. COGS de Roger da BE bruto 50-57% vs 11,7% operativo declarado.</t>
+          <t>AUTOSeg +100%→+50% · AUTOBulk +50%→+25%, si el escalón 1 contuvo sin frenar las permitidas.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -2394,7 +2295,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Bloquea comprar rank en heads con CVR probado</t>
+          <t>Depende del veredicto del guard del 17-ago</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -2416,52 +2317,334 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>AMC (Amazon Marketing Cloud)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Pedido de Roger en la meet: segmentación de audiencias. Instancia sin confirmar.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Resolvería el fallo del remarketing genérico</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>interno</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>5 keywords de test</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>NO LANZADAS. De 26 clusters solo 3 quedaron limpios y son débiles (SV 843-2.419).</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Diferido hasta refrescar el banco contra el bulk</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>interno</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BLOCKER · margen real</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Flete FBM no cargado por SKU. COGS de Roger da BE bruto 50-57% vs 11,7% operativo declarado.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Bloquea comprar rank en heads con CVR probado</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>interno</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
           <t>Hallazgo de ficha · B0CNVYVG9C</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>Serene 090x190 convierte 0,51% con Buy Box 94,5% y 197 sesiones.</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
         <is>
           <t>Problema de ficha, no de PPC. Revisar con Roger</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>interno</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Seguimiento</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Confirmar el efecto de los ajustes de la semana</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Los cambios de esta semana se miden a los siete días. El próximo lunes se confirma si el retorno mejoró y se decide si se amplían o se revierten.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>cliente</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Próxima fase</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Segmentación de audiencias</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Preparar la segmentación para dirigir la recuperación de visitantes a quienes ya mostraron interés en un producto concreto, en lugar de al catálogo completo.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>cliente</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Acción de catálogo</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Mejora de ficha de un modelo con baja conversión</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Un modelo de la gama principal recibe visitas pero convierte muy por debajo del resto. La disponibilidad está bien, así que la palanca está en la ficha del producto.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>cliente</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: fila MoM julio 2026 base SP+SB+SD (junio reproduce 12/12 columnas)
</commit_message>
<xml_diff>
--- a/pegar-sheet-W33/UPDATE-Sheet-W33.xlsx
+++ b/pegar-sheet-W33/UPDATE-Sheet-W33.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Acciones_PPC" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Bitacora" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Veredicto" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="MoM_KPIs" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2777,4 +2778,128 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Semana</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Ad_Sales</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ACoS</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ROAS</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>TACoS</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Ventas_Totales</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>CVR</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>BuyBox</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Impressions</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Clicks</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>CTR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>julio 2026</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3395.77</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23260.41</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.146</v>
+      </c>
+      <c r="E2" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G2" t="n">
+        <v>148</v>
+      </c>
+      <c r="H2" t="n">
+        <v>67907.49000000001</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.0198</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.9735</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1349851</v>
+      </c>
+      <c r="L2" t="n">
+        <v>6087</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.00451</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>